<commit_message>
fixed plot pricing and fixed upload
</commit_message>
<xml_diff>
--- a/import-templates/plot-import-template.xlsx
+++ b/import-templates/plot-import-template.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Template" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Instructions" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="Dropdown Values" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Instructions" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="35">
   <si>
     <t>project</t>
   </si>
@@ -50,25 +51,55 @@
     <t>available</t>
   </si>
   <si>
+    <t>A-101-2</t>
+  </si>
+  <si>
+    <t>blocked</t>
+  </si>
+  <si>
+    <t>Field (column)</t>
+  </si>
+  <si>
+    <t>Type exactly</t>
+  </si>
+  <si>
+    <t>Means (form label)</t>
+  </si>
+  <si>
+    <t>Vacant</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Not Vacant</t>
+  </si>
+  <si>
     <t>Column</t>
   </si>
   <si>
     <t>Required</t>
   </si>
   <si>
+    <t>Type</t>
+  </si>
+  <si>
     <t>Notes / valid values</t>
   </si>
   <si>
     <t>Yes</t>
   </si>
   <si>
+    <t>Text</t>
+  </si>
+  <si>
     <t>Existing project name (required, must match exactly)</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>Block / category name — created automatically if new</t>
+    <t>Block / category name (free text) — created automatically if new</t>
   </si>
   <si>
     <t>Plot number (required, unique within the project)</t>
@@ -77,13 +108,16 @@
     <t>Plot area in sq.ft (required, number &gt; 0)</t>
   </si>
   <si>
-    <t>₹ per sq.ft (optional, default 0)</t>
+    <t>₹ per sq.ft — drives plot value (optional, default 0). Value = sqft × this.</t>
   </si>
   <si>
     <t>Notes (optional)</t>
   </si>
   <si>
-    <t>available | blocked  (blocked = Not Vacant; default available)</t>
+    <t>Dropdown</t>
+  </si>
+  <si>
+    <t>Dropdown — type exactly: available (Vacant) or blocked (Not Vacant); default available</t>
   </si>
 </sst>
 </file>
@@ -102,12 +136,17 @@
       <b/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFF3F8"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -122,9 +161,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,35 +504,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="14" customWidth="1"/>
+    <col min="1" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -517,6 +557,29 @@
       </c>
       <c r="G2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3">
+        <v>1200</v>
+      </c>
+      <c r="E3">
+        <v>1500</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -527,100 +590,174 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="70" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="74" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>